<commit_message>
Enhance Dianghui protocol and GUI for XY sine control
- Updated the Dianghui protocol to support new command codes for sine wave generation on both X and Y axes.
- Introduced a new GUI component for simultaneous XY sine scanning, allowing users to set frequency and amplitude.
- Improved the handling of sine wave parameters, ensuring compatibility with the updated protocol.
- Adjusted the .gitignore to include additional Python files.
- Refactored existing methods for better clarity and performance in the control logic.
</commit_message>
<xml_diff>
--- a/开发协议/巅慧指令协议.xlsx
+++ b/开发协议/巅慧指令协议.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\28474\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\code\快反上位机\开发协议\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6238B90-3504-4019-A7ED-E637C12F6F2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285654E1-2034-4528-A155-F9F104631FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="指令帧" sheetId="1" r:id="rId1"/>
-    <sheet name="状态帧" sheetId="2" r:id="rId2"/>
+    <sheet name="正弦控制帧" sheetId="3" r:id="rId2"/>
+    <sheet name="状态帧" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="34">
   <si>
     <t>帧元</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -61,104 +62,115 @@
   </si>
   <si>
     <t>uint</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X轴设定值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y轴设定值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X轴限位值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y轴限位值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>保留</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>校验位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X轴使能状态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0:使能
+1:未使能</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y轴使能状态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自检状态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0:正常
+1:异常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X轴指令超限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0:未超限
+1:超限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y轴指令超限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y轴位置超限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X轴位置超限</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>通讯校验状态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>X轴位移监控</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y轴位移监控</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x0000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>正弦运动频率</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>正弦运动幅值</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>00:待命
 01:闭环
-04:开环
-05:自检</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X轴设定值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>int</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y轴设定值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X轴限位值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y轴限位值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>保留</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>校验位</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0x00</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X轴使能状态</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0:使能
-1:未使能</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y轴使能状态</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>自检状态</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0:正常
-1:异常</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X轴指令超限</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0:未超限
-1:超限</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y轴指令超限</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y轴位置超限</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X轴位置超限</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>通讯校验状态</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>X轴位移监控</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Y轴位移监控</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0x0000</t>
+02:自检
+03:开环
+04:快反镜X轴执行正弦扫描
+05:快反镜Y轴执行正弦扫描
+06:快反镜XY轴同时执行正弦扫描</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -487,120 +499,123 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A7:E15"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="57.9140625" customWidth="1"/>
+  </cols>
   <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="98" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+    </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="56" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14">
-        <v>8</v>
-      </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15">
-        <v>8</v>
-      </c>
-      <c r="C15" t="s">
         <v>8</v>
       </c>
     </row>
@@ -611,6 +626,135 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FBB5638-D38B-49E5-A19A-B9CB632BF94B}">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="98" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A0BF71D-3BC3-42D6-A1E9-83C89C7E9465}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
@@ -651,7 +795,7 @@
     </row>
     <row r="3" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -660,12 +804,12 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -674,12 +818,12 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -688,12 +832,12 @@
         <v>8</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -702,40 +846,40 @@
         <v>8</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -744,48 +888,48 @@
         <v>8</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11">
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13">
         <v>16</v>
@@ -794,12 +938,12 @@
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>8</v>

</xml_diff>